<commit_message>
Fix setting in EDA testing
</commit_message>
<xml_diff>
--- a/results/Int ACC.xlsx
+++ b/results/Int ACC.xlsx
@@ -878,52 +878,52 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>85.39 ± 4.52</t>
+          <t>85.11 ± 4.98</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>85.47 ± 4.77</t>
+          <t>85.25 ± 5.22</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>85.40 ± 4.77</t>
+          <t>85.15 ± 5.23</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>92.31 ± 5.40</t>
+          <t>92.40 ± 5.15</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>94.57 ± 3.73</t>
+          <t>94.60 ± 3.65</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>70.81 ± 9.40</t>
+          <t>70.33 ± 10.32</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>94.62 ± 3.64</t>
+          <t>94.63 ± 3.59</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>13.98 ± 5.85</t>
+          <t>14.24 ± 5.85</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>84.16 ± 8.88</t>
+          <t>83.83 ± 9.58</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>76.85 ± 12.43</t>
+          <t>76.77 ± 11.05</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -1310,52 +1310,52 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>85.89 ± 4.88</t>
+          <t>85.22 ± 5.07</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>85.98 ± 5.05</t>
+          <t>85.33 ± 5.34</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>85.91 ± 5.06</t>
+          <t>85.24 ± 5.34</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>92.46 ± 5.06</t>
+          <t>92.49 ± 4.94</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>94.70 ± 3.51</t>
+          <t>94.67 ± 3.45</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>71.82 ± 10.04</t>
+          <t>70.51 ± 10.54</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>94.72 ± 3.47</t>
+          <t>94.70 ± 3.41</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>14.26 ± 5.88</t>
+          <t>14.10 ± 6.01</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>83.33 ± 8.89</t>
+          <t>83.88 ± 8.87</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>77.14 ± 11.01</t>
+          <t>76.38 ± 12.10</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -1742,52 +1742,52 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>85.51 ± 4.88</t>
+          <t>85.60 ± 4.79</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>85.63 ± 5.13</t>
+          <t>85.69 ± 5.03</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>85.55 ± 5.13</t>
+          <t>85.63 ± 5.03</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>92.49 ± 5.21</t>
+          <t>92.60 ± 4.83</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>94.77 ± 3.43</t>
+          <t>94.78 ± 3.37</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>71.11 ± 10.14</t>
+          <t>71.24 ± 9.95</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>94.77 ± 3.43</t>
+          <t>94.79 ± 3.35</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>14.29 ± 5.54</t>
+          <t>14.07 ± 5.59</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>82.87 ± 9.28</t>
+          <t>84.05 ± 8.55</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>77.14 ± 10.80</t>
+          <t>77.45 ± 10.88</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -2174,52 +2174,52 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>86.21 ± 5.20</t>
+          <t>85.37 ± 5.39</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>86.28 ± 5.42</t>
+          <t>85.48 ± 5.55</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>86.20 ± 5.44</t>
+          <t>85.41 ± 5.56</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>92.49 ± 5.15</t>
+          <t>92.30 ± 5.11</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>94.74 ± 3.56</t>
+          <t>94.64 ± 3.49</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>72.44 ± 10.74</t>
+          <t>70.80 ± 11.05</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>94.75 ± 3.54</t>
+          <t>94.65 ± 3.48</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>13.83 ± 5.93</t>
+          <t>14.63 ± 5.75</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>84.20 ± 9.10</t>
+          <t>83.07 ± 9.60</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>77.31 ± 11.23</t>
+          <t>76.71 ± 11.77</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
@@ -2606,52 +2606,52 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>85.73 ± 4.79</t>
+          <t>85.53 ± 4.61</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>85.84 ± 5.00</t>
+          <t>85.63 ± 4.80</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>85.77 ± 5.01</t>
+          <t>85.56 ± 4.80</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>92.35 ± 5.35</t>
+          <t>92.51 ± 5.04</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>94.71 ± 3.55</t>
+          <t>94.76 ± 3.43</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>71.53 ± 9.91</t>
+          <t>71.11 ± 9.52</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>94.72 ± 3.53</t>
+          <t>94.79 ± 3.39</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>13.93 ± 5.66</t>
+          <t>13.99 ± 5.77</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>83.76 ± 9.27</t>
+          <t>84.54 ± 8.70</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>77.51 ± 11.28</t>
+          <t>77.08 ± 10.84</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
@@ -3038,52 +3038,52 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>84.96 ± 3.47</t>
+          <t>85.02 ± 4.03</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>84.99 ± 3.55</t>
+          <t>85.06 ± 4.10</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>84.90 ± 3.57</t>
+          <t>84.97 ± 4.13</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>92.30 ± 3.67</t>
+          <t>92.35 ± 3.55</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>94.53 ± 2.45</t>
+          <t>94.55 ± 2.35</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>69.86 ± 7.02</t>
+          <t>69.99 ± 8.13</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>94.55 ± 2.43</t>
+          <t>94.56 ± 2.34</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>14.52 ± 3.53</t>
+          <t>14.77 ± 4.32</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>80.29 ± 9.04</t>
+          <t>80.42 ± 8.44</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>74.32 ± 8.59</t>
+          <t>74.76 ± 7.22</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
@@ -3470,52 +3470,52 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>84.41 ± 5.36</t>
+          <t>84.94 ± 4.92</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>84.45 ± 5.50</t>
+          <t>84.95 ± 5.09</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>84.42 ± 5.49</t>
+          <t>84.92 ± 5.08</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>91.57 ± 4.81</t>
+          <t>91.79 ± 4.75</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>94.05 ± 3.07</t>
+          <t>94.26 ± 3.08</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>68.81 ± 10.95</t>
+          <t>69.83 ± 10.10</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>94.05 ± 3.08</t>
+          <t>94.27 ± 3.06</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>15.60 ± 5.78</t>
+          <t>14.75 ± 5.40</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>80.32 ± 10.36</t>
+          <t>82.28 ± 9.69</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>75.40 ± 9.44</t>
+          <t>76.83 ± 9.98</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
@@ -3902,52 +3902,52 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>84.27 ± 6.42</t>
+          <t>83.96 ± 5.94</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>84.22 ± 6.56</t>
+          <t>83.93 ± 6.08</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>84.14 ± 6.66</t>
+          <t>83.86 ± 6.16</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>91.17 ± 5.01</t>
+          <t>91.24 ± 4.94</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>93.26 ± 3.56</t>
+          <t>93.40 ± 3.59</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>68.47 ± 12.97</t>
+          <t>67.87 ± 12.01</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>93.30 ± 3.59</t>
+          <t>93.41 ± 3.60</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>15.47 ± 5.92</t>
+          <t>15.41 ± 5.73</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>80.19 ± 10.87</t>
+          <t>80.25 ± 10.49</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>73.38 ± 12.29</t>
+          <t>73.63 ± 11.90</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
@@ -4334,52 +4334,52 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>84.43 ± 5.60</t>
+          <t>84.85 ± 4.67</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>84.27 ± 5.64</t>
+          <t>84.67 ± 4.74</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>84.20 ± 5.68</t>
+          <t>84.60 ± 4.78</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>91.27 ± 5.41</t>
+          <t>91.48 ± 5.15</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>93.54 ± 3.37</t>
+          <t>93.59 ± 3.25</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>68.62 ± 11.26</t>
+          <t>69.44 ± 9.44</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>93.55 ± 3.36</t>
+          <t>93.61 ± 3.23</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>16.06 ± 6.27</t>
+          <t>15.94 ± 5.95</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>80.81 ± 8.39</t>
+          <t>80.88 ± 8.26</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>74.46 ± 6.98</t>
+          <t>74.97 ± 7.71</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
@@ -4766,52 +4766,52 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>86.48 ± 6.71</t>
+          <t>86.35 ± 6.80</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>86.78 ± 6.28</t>
+          <t>86.63 ± 6.42</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>86.57 ± 6.55</t>
+          <t>86.43 ± 6.66</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>93.27 ± 5.37</t>
+          <t>93.02 ± 5.40</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>94.01 ± 4.73</t>
+          <t>93.87 ± 4.61</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>73.19 ± 12.97</t>
+          <t>72.91 ± 13.22</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>94.01 ± 4.72</t>
+          <t>93.87 ± 4.61</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>13.28 ± 7.35</t>
+          <t>13.82 ± 7.59</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>81.46 ± 13.20</t>
+          <t>80.80 ± 12.87</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>76.54 ± 13.65</t>
+          <t>76.50 ± 13.45</t>
         </is>
       </c>
       <c r="O41" t="inlineStr">
@@ -5198,52 +5198,52 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>86.87 ± 6.25</t>
+          <t>87.27 ± 6.53</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>87.14 ± 6.01</t>
+          <t>87.51 ± 6.27</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>86.98 ± 6.18</t>
+          <t>87.36 ± 6.43</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>93.57 ± 4.66</t>
+          <t>93.83 ± 4.51</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>94.20 ± 4.22</t>
+          <t>94.48 ± 3.96</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>74.00 ± 12.23</t>
+          <t>74.76 ± 12.74</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>94.20 ± 4.22</t>
+          <t>94.48 ± 3.96</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>13.37 ± 6.58</t>
+          <t>12.84 ± 6.66</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>82.86 ± 11.68</t>
+          <t>82.78 ± 11.87</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>77.66 ± 14.49</t>
+          <t>78.12 ± 15.16</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
@@ -5630,52 +5630,52 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>85.94 ± 8.71</t>
+          <t>86.03 ± 8.93</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>86.87 ± 7.68</t>
+          <t>86.87 ± 7.81</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>86.61 ± 8.18</t>
+          <t>86.60 ± 8.34</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>92.55 ± 8.86</t>
+          <t>92.60 ± 9.14</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>91.98 ± 8.81</t>
+          <t>92.21 ± 8.84</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>72.39 ± 16.79</t>
+          <t>72.40 ± 17.12</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>92.00 ± 8.77</t>
+          <t>92.24 ± 8.78</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>13.57 ± 10.30</t>
+          <t>13.23 ± 10.58</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>81.34 ± 17.80</t>
+          <t>81.38 ± 18.20</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>74.54 ± 19.81</t>
+          <t>75.17 ± 20.03</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
@@ -6062,52 +6062,52 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>87.17 ± 7.03</t>
+          <t>86.67 ± 7.33</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>88.47 ± 6.02</t>
+          <t>88.08 ± 6.36</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>88.29 ± 6.21</t>
+          <t>87.88 ± 6.56</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>92.32 ± 8.38</t>
+          <t>92.20 ± 8.58</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>91.81 ± 7.54</t>
+          <t>91.80 ± 7.65</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>75.06 ± 13.50</t>
+          <t>74.18 ± 14.23</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>91.85 ± 7.52</t>
+          <t>91.82 ± 7.63</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>14.00 ± 9.47</t>
+          <t>14.11 ± 9.47</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>82.61 ± 14.26</t>
+          <t>82.95 ± 14.42</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>78.52 ± 15.25</t>
+          <t>79.13 ± 15.61</t>
         </is>
       </c>
       <c r="O53" t="inlineStr">
@@ -6494,52 +6494,52 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>87.68 ± 8.21</t>
+          <t>87.60 ± 8.17</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>89.04 ± 6.08</t>
+          <t>89.14 ± 6.02</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>88.65 ± 6.99</t>
+          <t>88.72 ± 6.96</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>92.31 ± 10.05</t>
+          <t>92.52 ± 9.28</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>91.11 ± 9.69</t>
+          <t>91.24 ± 9.37</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>75.60 ± 15.08</t>
+          <t>75.72 ± 15.02</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>91.11 ± 9.69</t>
+          <t>91.25 ± 9.33</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>13.92 ± 10.37</t>
+          <t>13.74 ± 10.26</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>81.44 ± 15.99</t>
+          <t>81.20 ± 15.83</t>
         </is>
       </c>
       <c r="N57" t="inlineStr">
         <is>
-          <t>76.40 ± 18.25</t>
+          <t>75.47 ± 17.51</t>
         </is>
       </c>
       <c r="O57" t="inlineStr">
@@ -6926,52 +6926,52 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>84.72 ± 7.79</t>
+          <t>84.72 ± 7.38</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>88.21 ± 4.68</t>
+          <t>88.24 ± 4.28</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>87.78 ± 5.21</t>
+          <t>87.81 ± 4.82</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>91.44 ± 9.37</t>
+          <t>91.35 ± 9.09</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>88.92 ± 9.52</t>
+          <t>88.65 ± 9.62</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>70.89 ± 13.10</t>
+          <t>70.98 ± 12.23</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>88.96 ± 9.44</t>
+          <t>88.69 ± 9.53</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>14.76 ± 10.33</t>
+          <t>15.35 ± 10.78</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>82.11 ± 14.67</t>
+          <t>81.28 ± 15.47</t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t>74.00 ± 14.72</t>
+          <t>73.84 ± 15.15</t>
         </is>
       </c>
       <c r="O61" t="inlineStr">
@@ -7358,52 +7358,52 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>83.82 ± 10.26</t>
+          <t>83.67 ± 9.80</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>88.88 ± 5.51</t>
+          <t>88.77 ± 5.41</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>88.27 ± 6.29</t>
+          <t>88.19 ± 6.14</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>90.06 ± 11.97</t>
+          <t>90.08 ± 11.97</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>86.37 ± 13.91</t>
+          <t>86.35 ± 13.75</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>69.14 ± 17.15</t>
+          <t>69.01 ± 16.63</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>86.36 ± 13.93</t>
+          <t>86.33 ± 13.78</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>16.83 ± 13.08</t>
+          <t>16.74 ± 13.43</t>
         </is>
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>78.41 ± 18.67</t>
+          <t>78.36 ± 18.82</t>
         </is>
       </c>
       <c r="N65" t="inlineStr">
         <is>
-          <t>75.07 ± 20.46</t>
+          <t>75.36 ± 20.24</t>
         </is>
       </c>
       <c r="O65" t="inlineStr">
@@ -7790,52 +7790,52 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>83.89 ± 13.45</t>
+          <t>82.69 ± 14.12</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>90.48 ± 6.63</t>
+          <t>89.72 ± 7.06</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>89.68 ± 8.19</t>
+          <t>88.83 ± 8.61</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>88.51 ± 18.08</t>
+          <t>89.22 ± 17.14</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>83.50 ± 21.98</t>
+          <t>83.72 ± 21.92</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>68.85 ± 25.87</t>
+          <t>66.38 ± 26.97</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>83.20 ± 22.81</t>
+          <t>83.48 ± 22.60</t>
         </is>
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>17.06 ± 17.33</t>
+          <t>16.39 ± 17.17</t>
         </is>
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>78.52 ± 25.63</t>
+          <t>78.63 ± 26.39</t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
         <is>
-          <t>73.47 ± 27.81</t>
+          <t>72.43 ± 28.83</t>
         </is>
       </c>
       <c r="O69" t="inlineStr">
@@ -8222,52 +8222,52 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>84.77 ± 15.94</t>
+          <t>85.13 ± 15.70</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>92.32 ± 7.23</t>
+          <t>92.24 ± 7.58</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>91.39 ± 9.13</t>
+          <t>91.42 ± 9.46</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>92.45 ± 16.43</t>
+          <t>92.55 ± 16.78</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>85.53 ± 23.72</t>
+          <t>85.34 ± 24.41</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>70.10 ± 31.13</t>
+          <t>70.63 ± 31.36</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>85.27 ± 24.33</t>
+          <t>85.04 ± 25.08</t>
         </is>
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>12.22 ± 16.94</t>
+          <t>11.33 ± 16.98</t>
         </is>
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>85.74 ± 23.27</t>
+          <t>86.36 ± 24.69</t>
         </is>
       </c>
       <c r="N73" t="inlineStr">
         <is>
-          <t>78.03 ± 30.94</t>
+          <t>78.94 ± 32.38</t>
         </is>
       </c>
       <c r="O73" t="inlineStr">
@@ -8654,52 +8654,52 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>85.47 ± 16.38</t>
+          <t>86.13 ± 15.41</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>93.02 ± 7.38</t>
+          <t>93.18 ± 7.33</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>92.10 ± 9.32</t>
+          <t>92.42 ± 9.01</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>91.76 ± 18.37</t>
+          <t>91.61 ± 18.81</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>84.74 ± 26.78</t>
+          <t>84.52 ± 26.44</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>72.14 ± 32.39</t>
+          <t>73.57 ± 30.41</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>84.42 ± 27.50</t>
+          <t>84.16 ± 27.25</t>
         </is>
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>11.29 ± 17.95</t>
+          <t>11.79 ± 17.95</t>
         </is>
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>83.22 ± 28.76</t>
+          <t>84.43 ± 27.48</t>
         </is>
       </c>
       <c r="N77" t="inlineStr">
         <is>
-          <t>79.63 ± 32.92</t>
+          <t>79.48 ± 33.26</t>
         </is>
       </c>
       <c r="O77" t="inlineStr">
@@ -9086,52 +9086,52 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>85.67 ± 15.43</t>
+          <t>85.27 ± 16.29</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>93.59 ± 6.55</t>
+          <t>93.43 ± 6.80</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>92.55 ± 8.63</t>
+          <t>92.20 ± 9.38</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>93.45 ± 14.59</t>
+          <t>93.76 ± 13.46</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>87.64 ± 19.44</t>
+          <t>86.49 ± 20.76</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>72.77 ± 28.51</t>
+          <t>71.43 ± 31.18</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>87.45 ± 19.85</t>
+          <t>86.42 ± 20.88</t>
         </is>
       </c>
       <c r="L81" t="inlineStr">
         <is>
-          <t>10.18 ± 15.23</t>
+          <t>9.91 ± 14.04</t>
         </is>
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>89.14 ± 21.66</t>
+          <t>88.75 ± 21.88</t>
         </is>
       </c>
       <c r="N81" t="inlineStr">
         <is>
-          <t>85.28 ± 21.80</t>
+          <t>83.45 ± 24.03</t>
         </is>
       </c>
       <c r="O81" t="inlineStr">
@@ -9518,52 +9518,52 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>85.05 ± 16.89</t>
+          <t>84.61 ± 16.75</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>93.44 ± 6.53</t>
+          <t>93.21 ± 6.25</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>92.16 ± 9.36</t>
+          <t>91.97 ± 8.86</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>93.34 ± 13.80</t>
+          <t>92.89 ± 15.09</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>75.91 ± 30.45</t>
+          <t>76.58 ± 30.70</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>60.88 ± 36.80</t>
+          <t>59.85 ± 35.80</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
         <is>
-          <t>80.84 ± 19.81</t>
+          <t>81.37 ± 20.38</t>
         </is>
       </c>
       <c r="L85" t="inlineStr">
         <is>
-          <t>19.35 ± 30.09</t>
+          <t>19.69 ± 30.48</t>
         </is>
       </c>
       <c r="M85" t="inlineStr">
         <is>
-          <t>87.96 ± 21.71</t>
+          <t>87.96 ± 21.94</t>
         </is>
       </c>
       <c r="N85" t="inlineStr">
         <is>
-          <t>80.31 ± 25.42</t>
+          <t>80.64 ± 23.20</t>
         </is>
       </c>
       <c r="O85" t="inlineStr">

</xml_diff>